<commit_message>
feat: update sample data to real-world (NXX) NXX-XXXX phone format
- generate_sample.js: phone numbers now use (813) 767-1412 style matching
  real ENS report exports from hospital systems
- Added PCP column, 4 patients, Florida-area codes for realistic testing
- Regenerated sample.xlsx with the new format
- WorkflowEngine already handles this format correctly via /\D/g stripping
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -428,12 +428,15 @@
         <v>Practice Name</v>
       </c>
       <c r="J1" t="str">
+        <v>PCP</v>
+      </c>
+      <c r="K1" t="str">
         <v>Cell Phone</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Home Phone</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Work Phone</v>
       </c>
     </row>
@@ -460,18 +463,21 @@
         <v>Inpatient</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-22</v>
       </c>
       <c r="I2" t="str">
         <v>Valley Health Center</v>
       </c>
       <c r="J2" t="str">
-        <v>5551234567</v>
+        <v>Dr. Sarah Smith</v>
       </c>
       <c r="K2" t="str">
-        <v>5559876543</v>
+        <v>(813) 767-1412</v>
       </c>
       <c r="L2" t="str">
+        <v>(813) 555-9876</v>
+      </c>
+      <c r="M2" t="str">
         <v/>
       </c>
     </row>
@@ -498,24 +504,109 @@
         <v>Inpatient</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-22</v>
       </c>
       <c r="I3" t="str">
         <v>Apex Medical Group</v>
       </c>
       <c r="J3" t="str">
+        <v>Dr. Marcus Brown</v>
+      </c>
+      <c r="K3" t="str">
         <v/>
       </c>
-      <c r="K3" t="str">
-        <v>5558000143</v>
-      </c>
       <c r="L3" t="str">
+        <v>(727) 800-0143</v>
+      </c>
+      <c r="M3" t="str">
         <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>MRN-512</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Marcus</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Watney</v>
+      </c>
+      <c r="D4" t="str">
+        <v>1975-03-22</v>
+      </c>
+      <c r="E4" t="str">
+        <v>M</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Discharge</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Inpatient</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2026-06-22</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Bay Area Health</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Dr. Elena Rostova</v>
+      </c>
+      <c r="K4" t="str">
+        <v>(407) 303-4920</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>MRN-774</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Diana</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Prince</v>
+      </c>
+      <c r="D5" t="str">
+        <v>1990-07-04</v>
+      </c>
+      <c r="E5" t="str">
+        <v>F</v>
+      </c>
+      <c r="F5" t="str">
+        <v>End Visit</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Inpatient</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-06-22</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Sunrise Medical Center</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Dr. Sarah Smith</v>
+      </c>
+      <c r="K5" t="str">
+        <v>(954) 444-5555</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v>(954) 444-9900</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>